<commit_message>
Add Mean_NRMSE and cation/anion group aggregates to error metrics
Both error-calculation scripts now persist Mean_NRMSE_% in their
per-group and overall aggregate sections; previously only per-row
NRMSE_% was reported, so cross-species and cross-case comparison
required computing the means by hand.

The cation-exchange script also gains a METRICS_BY_GROUP section
(text report + Excel sheet) reporting RMSE, NRMSE, R^2, NSE, etc.
for cations (Ca2+, Na+, K+) and anions (Cl-, NO3-) separately. The
cation-only mean NRMSE (~2%) is what the reactive-transport
benchmark is actually testing; the anion mean is inflated by a
near-depleted Day 3 NO3- row (N=5) and should not be the headline
number.

Regenerated .txt and .xlsx outputs in both ANALYSIS_AND_FIGURES
folders. Removed obsolete ERROR.xlsx (superseded by
RESULTS_CATION_EXCHANGE_ERROR_METRICS.xlsx) and updated the
matching README references.

Co-Authored-By: Claude Opus 4.7 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/1_BENCHMARKING_STUDY/ANALYSIS_AND_FIGURES/RESULTS_BENCHMARKING_ERROR_METRICS.xlsx
+++ b/1_BENCHMARKING_STUDY/ANALYSIS_AND_FIGURES/RESULTS_BENCHMARKING_ERROR_METRICS.xlsx
@@ -789,7 +789,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I4"/>
+  <dimension ref="A1:J4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -815,25 +815,30 @@
       </c>
       <c r="E1" t="inlineStr">
         <is>
+          <t>Mean_NRMSE_%</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
           <t>Mean_MAE</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>Max_AbsError</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>Max_AbsError_DAY</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>Mean_R2</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>Mean_NSE</t>
         </is>
@@ -855,18 +860,21 @@
         <v>0.0006687879880998262</v>
       </c>
       <c r="E2" t="n">
+        <v>0.05024653864860202</v>
+      </c>
+      <c r="F2" t="n">
         <v>0.0003254272456510972</v>
       </c>
-      <c r="F2" t="n">
+      <c r="G2" t="n">
         <v>0.007591104053714149</v>
       </c>
-      <c r="G2" t="n">
-        <v>3</v>
-      </c>
       <c r="H2" t="n">
+        <v>3</v>
+      </c>
+      <c r="I2" t="n">
         <v>0.9999982945499587</v>
       </c>
-      <c r="I2" t="n">
+      <c r="J2" t="n">
         <v>0.9999958886470607</v>
       </c>
     </row>
@@ -886,18 +894,21 @@
         <v>0.0006545188291307876</v>
       </c>
       <c r="E3" t="n">
+        <v>0.06446025486581039</v>
+      </c>
+      <c r="F3" t="n">
         <v>0.0004762500285313607</v>
       </c>
-      <c r="F3" t="n">
+      <c r="G3" t="n">
         <v>0.003830989096417567</v>
       </c>
-      <c r="G3" t="n">
-        <v>3</v>
-      </c>
       <c r="H3" t="n">
+        <v>3</v>
+      </c>
+      <c r="I3" t="n">
         <v>0.999999350053043</v>
       </c>
-      <c r="I3" t="n">
+      <c r="J3" t="n">
         <v>0.9999956058813838</v>
       </c>
     </row>
@@ -917,18 +928,21 @@
         <v>0.0009306669087837991</v>
       </c>
       <c r="E4" t="n">
+        <v>0.1030513667682624</v>
+      </c>
+      <c r="F4" t="n">
         <v>0.0008049281032395484</v>
       </c>
-      <c r="F4" t="n">
+      <c r="G4" t="n">
         <v>0.002597485274327405</v>
       </c>
-      <c r="G4" t="n">
-        <v>3</v>
-      </c>
       <c r="H4" t="n">
+        <v>3</v>
+      </c>
+      <c r="I4" t="n">
         <v>0.9999979463022449</v>
       </c>
-      <c r="I4" t="n">
+      <c r="J4" t="n">
         <v>0.9999894021327087</v>
       </c>
     </row>
@@ -943,7 +957,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G2"/>
+  <dimension ref="A1:H2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -964,20 +978,25 @@
       </c>
       <c r="D1" t="inlineStr">
         <is>
+          <t>Mean_NRMSE_%</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
           <t>Mean_MAE</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>Max_AbsError</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>Mean_R2</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>Mean_NSE</t>
         </is>
@@ -994,15 +1013,18 @@
         <v>0.0007619740078284698</v>
       </c>
       <c r="D2" t="n">
+        <v>0.07258605342755829</v>
+      </c>
+      <c r="E2" t="n">
         <v>0.0005355351258073354</v>
       </c>
-      <c r="E2" t="n">
+      <c r="F2" t="n">
         <v>0.007591104053714149</v>
       </c>
-      <c r="F2" t="n">
+      <c r="G2" t="n">
         <v>0.9999985303017487</v>
       </c>
-      <c r="G2" t="n">
+      <c r="H2" t="n">
         <v>0.9999936322203844</v>
       </c>
     </row>

</xml_diff>